<commit_message>
worker_09: mark the cooldown case manual by design
The cooldown only exists for a real registered number and every invite/resend
texts it, so the invite cannot be refreshed on each CI run without texting a real
person (demo numbers send no SMS, so they never enforce the cooldown). The test
stays and verifies the refusal while a manually refreshed invite is <24h old;
otherwise it skips, now saying so. MTP rows updated to match.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Web_Platform_MTP.xlsx
+++ b/test_plans/CCC_Web_Platform_MTP.xlsx
@@ -3645,7 +3645,7 @@
       <c r="F12" s="85" t="n"/>
       <c r="G12" s="88" t="inlineStr">
         <is>
-          <t>✅ Automated (Playwright): test_worker_lifecycle.py::test_connect_worker_09_resend_cooldown (real number +919000696488 -&gt; "sent in the last 24 hours"). NOTE: relies on the invite staying &lt;24h old; refresh if it flips.</t>
+          <t>🟡 Manual by design (decided 2026-10-02): the cooldown only exists for a real registered number and every invite/resend texts it, so it cannot be refreshed on each CI run without texting a real person (demo numbers send no SMS, so they never enforce the cooldown). test_worker_lifecycle.py::test_connect_worker_09_resend_cooldown (+919000696488, "sent in the last 24 hours") still verifies the refusal whenever the invite is &lt;24h old, e.g. right after a manual re-invite; otherwise it skips without resending. Run manually before releases.</t>
         </is>
       </c>
     </row>
@@ -32970,7 +32970,7 @@
       </c>
       <c r="D338" s="171" t="inlineStr">
         <is>
-          <t>🟢 Already automated</t>
+          <t>🟡 Manual by design</t>
         </is>
       </c>
       <c r="E338" s="171" t="inlineStr">
@@ -32985,7 +32985,7 @@
       </c>
       <c r="G338" s="171" t="inlineStr">
         <is>
-          <t>Already automated (n/a)</t>
+          <t>QA-owned (manual) - real-number cooldown; the test skips when the invite is &gt;24h old</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
MTP: tidy the old worker_09/worker_10 gap rows
GAP-CW-07 (worker_09) now reads Manual only (by design), pointing at the automated
test that stays manual-by-design; GAP-CW-08 (worker_10) is closed as already
automated. worker_09 sits in the dashboard's Manual only bucket (red), not
Automatable-not-built (yellow), since the Dashboard counts by status prefix.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Web_Platform_MTP.xlsx
+++ b/test_plans/CCC_Web_Platform_MTP.xlsx
@@ -24978,12 +24978,12 @@
       </c>
       <c r="D122" s="171" t="inlineStr">
         <is>
-          <t>🔴 Manual only</t>
+          <t>🔴 Manual only (by design)</t>
         </is>
       </c>
       <c r="E122" s="171" t="inlineStr">
         <is>
-          <t>24-hr cooldown - time-dependent</t>
+          <t>Superseded: an automated test exists (Connect_worker_09, test_worker_lifecycle.py::test_connect_worker_09_resend_cooldown) but is manual by design - the cooldown needs a real registered number and every invite/resend texts it, so the invite cannot be refreshed on each CI run</t>
         </is>
       </c>
       <c r="F122" s="171" t="inlineStr">
@@ -25015,12 +25015,12 @@
       </c>
       <c r="D123" s="171" t="inlineStr">
         <is>
-          <t>🔴 Manual only</t>
+          <t>🟢 Already automated</t>
         </is>
       </c>
       <c r="E123" s="171" t="inlineStr">
         <is>
-          <t>24-hr cooldown - time-dependent</t>
+          <t>Closed: automated as Connect_worker_10, test_worker_lifecycle.py::test_connect_worker_10_resend_allowed_for_pending (seeded data, Worker_Lifecycle_Automation, 2026-09-10)</t>
         </is>
       </c>
       <c r="F123" s="171" t="inlineStr">
@@ -25030,7 +25030,7 @@
       </c>
       <c r="G123" s="171" t="inlineStr">
         <is>
-          <t>QA-owned (manual)</t>
+          <t>Already automated (n/a)</t>
         </is>
       </c>
     </row>
@@ -32970,7 +32970,7 @@
       </c>
       <c r="D338" s="171" t="inlineStr">
         <is>
-          <t>🟡 Manual by design</t>
+          <t>🔴 Manual only (by design)</t>
         </is>
       </c>
       <c r="E338" s="171" t="inlineStr">

</xml_diff>

<commit_message>
MTP: update VV_31-35 and GAP-40/42/43 comments for the self-seeding review tests
Mark VV_31-34 as running on prod + staging with self-topped-up data, split VV_35 into the passing
agree-then-cannot-disagree half and the expected-failure half (product leaves Agree enabled after
Disagree), and note GAP-40/GAP-43-NM skip because the seeded opps have WORKER_VISITS_TASKS ON.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Web_Platform_MTP.xlsx
+++ b/test_plans/CCC_Web_Platform_MTP.xlsx
@@ -5872,7 +5872,7 @@
       <c r="F33" s="87" t="n"/>
       <c r="G33" s="73" t="inlineStr">
         <is>
-          <t>This test is for opp created before june 2 | ✅ Automated: test_vv_31_nm_reject_visit (NM org). Skips until a seeded manual-review opp with pending visits exists.</t>
+          <t>This test is for opp created before june 2 | ✅ Automated: test_vv_31_nm_reject_visit (NM org). Runs on prod and staging against the seeded 'Manual approval opp'. The tests top up their own pool of visits by submitting the delivery form in HQ Web Apps as the worker ('Log in as'), so no manual reseeding.</t>
         </is>
       </c>
     </row>
@@ -5903,7 +5903,7 @@
       <c r="F34" s="87" t="n"/>
       <c r="G34" s="73" t="inlineStr">
         <is>
-          <t>This test is for opp created before june 3 | ✅ Automated: test_vv_32_nm_approve_visit (NM org). Skips until a seeded manual-review opp with pending visits exists.</t>
+          <t>This test is for opp created before june 3 | ✅ Automated: test_vv_32_nm_approve_visit (NM org). Runs on prod and staging against the seeded 'Manual approval opp'. The tests top up their own pool of visits by submitting the delivery form in HQ Web Apps as the worker ('Log in as'), so no manual reseeding.</t>
         </is>
       </c>
     </row>
@@ -5934,7 +5934,7 @@
       <c r="F35" s="87" t="n"/>
       <c r="G35" s="73" t="inlineStr">
         <is>
-          <t>This test is for opp created before june 4 | ✅ Automated: test_vv_33_pm_agree_visit. Skips until seeded NM-approved / PM-review-pending visits exist.</t>
+          <t>This test is for opp created before june 4 | ✅ Automated: test_vv_33_pm_agree_visit. Runs on prod and staging against the seeded 'Manual approval opp'. The tests top up their own pool of visits by submitting the delivery form in HQ Web Apps as the worker ('Log in as'), so no manual reseeding. PM-review-pending visits come from the fixture NM-approving fresh visits.</t>
         </is>
       </c>
     </row>
@@ -5965,7 +5965,7 @@
       <c r="F36" s="87" t="n"/>
       <c r="G36" s="73" t="inlineStr">
         <is>
-          <t>This test is for opp created before june 5 | ✅ Automated: test_vv_34_pm_disagree_visit. Skips until seeded NM-approved / PM-review-pending visits exist.</t>
+          <t>This test is for opp created before june 5 | ✅ Automated: test_vv_34_pm_disagree_visit. Runs on prod and staging against the seeded 'Manual approval opp'. The tests top up their own pool of visits by submitting the delivery form in HQ Web Apps as the worker ('Log in as'), so no manual reseeding. PM-review-pending visits come from the fixture NM-approving fresh visits.</t>
         </is>
       </c>
     </row>
@@ -5986,7 +5986,7 @@
       <c r="F37" s="87" t="n"/>
       <c r="G37" s="73" t="inlineStr">
         <is>
-          <t>✅ Automated: test_vv_35_agree_and_disagree_are_mutually_exclusive (disagreed visit can't be agreed &amp; vice-versa). Skips until manual-review opp seeded.</t>
+          <t>✅ Automated, split in two: test_vv_35_agree_then_cannot_disagree PASSES (after Agree, Disagree is disabled). test_vv_35_disagree_then_cannot_agree is an EXPECTED FAILURE (xfail): the product leaves Agree enabled after Disagree (Agree is only disabled once the visit is already agreed), so a PM can flip disagree -&gt; agree, which contradicts this case. Product bug or plan inaccuracy - decision pending (seen on prod and staging, 2026-10-16).</t>
         </is>
       </c>
     </row>
@@ -6244,7 +6244,7 @@
       <c r="F47" s="73" t="inlineStr"/>
       <c r="G47" s="73" t="inlineStr">
         <is>
-          <t>✅ Automated: test_gap_w_40_verification_tab_set_by_mode_and_role. Asserts PM sees Pending PM Review (not Pending NM Review), NM sees both, set ends with 'All'. Skips until manual-review opp seeded / when WORKER_VISITS_TASKS switch ON.</t>
+          <t>✅ Automated: test_gap_w_40_verification_tab_set_by_mode_and_role. Asserts PM sees Pending PM Review (not Pending NM Review), NM sees both, set ends with 'All'. Currently SKIPS on prod and staging: the seeded manual-review opps have the WORKER_VISITS_TASKS switch ON (plain Visits/Tasks table, no NM-review tab-set); needs an opp with the switch OFF.</t>
         </is>
       </c>
     </row>
@@ -6286,7 +6286,7 @@
       <c r="F49" s="73" t="inlineStr"/>
       <c r="G49" s="73" t="inlineStr">
         <is>
-          <t>✅ Automated (partial): test_gap_w_42_reject_requires_reason + test_gap_w_42_approve_requires_justification (mandatory reason/justification enforced). 100-visit bulk cap NOT covered (needs &gt;100 seeded visits).</t>
+          <t>✅ Automated (partial): test_gap_w_42_reject_requires_reason + test_gap_w_42_approve_requires_justification - both passing on prod and staging (the reject textarea has no 'required' attribute, but the server refuses an empty reason; approve's justification is required client-side). 100-visit bulk cap NOT covered (needs &gt;100 seeded visits).</t>
         </is>
       </c>
     </row>
@@ -6307,7 +6307,7 @@
       <c r="F50" s="73" t="inlineStr"/>
       <c r="G50" s="73" t="inlineStr">
         <is>
-          <t>✅ Automated: test_gap_w_43_bulk_controls_hidden_for_pm (passing). NM positive control test_gap_w_43_bulk_controls_visible_for_nm skips until a seeded manual-review opp.</t>
+          <t>✅ Automated: test_gap_w_43_bulk_controls_hidden_for_pm (passing). NM positive control test_gap_w_43_bulk_controls_visible_for_nm SKIPS: bulk controls belong to the tabbed verification table, which is absent when the WORKER_VISITS_TASKS switch is ON (the case on the seeded opps).</t>
         </is>
       </c>
     </row>

</xml_diff>